<commit_message>
added comparison of cards
</commit_message>
<xml_diff>
--- a/ms_teams_copilot_client_answers.xlsx
+++ b/ms_teams_copilot_client_answers.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MohitVerma\Desktop\git\translation\SaS-to-python\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB645F27-3797-4993-964A-D9DD09B5FAFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BAE94EB-60A4-423B-B914-5A266A83621C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Quick Summary" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="169">
   <si>
     <t>Quick summary for the client</t>
   </si>
@@ -664,6 +664,33 @@
  Summarize insights in 1–2 paragraphs highlighting what drives discussion volume (e.g., promotions, rate cuts, scandals, or UX)._x000D_
 _x000D_
 Return the final output as a **Markdown table**. _x000D_</t>
+  </si>
+  <si>
+    <t>Jp Morgan</t>
+  </si>
+  <si>
+    <t>Amex</t>
+  </si>
+  <si>
+    <t>Citi</t>
+  </si>
+  <si>
+    <t>Bank of America</t>
+  </si>
+  <si>
+    <t>Wells Fargo</t>
+  </si>
+  <si>
+    <t>US Bank</t>
+  </si>
+  <si>
+    <t>Goldman Sachs</t>
+  </si>
+  <si>
+    <t>USAA</t>
+  </si>
+  <si>
+    <t>PNC Bank</t>
   </si>
 </sst>
 </file>
@@ -811,7 +838,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -849,6 +876,7 @@
     <xf numFmtId="15" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" readingOrder="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -859,7 +887,12 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2400,22 +2433,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
     </row>
     <row r="2" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
     </row>
     <row r="4" spans="1:5" ht="26" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
@@ -2613,40 +2646,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
     </row>
     <row r="2" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="16"/>
-      <c r="H2" s="16"/>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="17"/>
+      <c r="H2" s="17"/>
     </row>
     <row r="3" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="15" t="s">
+      <c r="A3" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="B3" s="16"/>
-      <c r="C3" s="16"/>
-      <c r="D3" s="16"/>
-      <c r="E3" s="16"/>
-      <c r="F3" s="16"/>
-      <c r="G3" s="16"/>
-      <c r="H3" s="16"/>
+      <c r="B3" s="17"/>
+      <c r="C3" s="17"/>
+      <c r="D3" s="17"/>
+      <c r="E3" s="17"/>
+      <c r="F3" s="17"/>
+      <c r="G3" s="17"/>
+      <c r="H3" s="17"/>
     </row>
     <row r="4" spans="1:8" ht="26" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
@@ -2932,24 +2965,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="18" t="s">
         <v>94</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
     </row>
     <row r="2" spans="1:6" ht="42" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="16" t="s">
         <v>95</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
     </row>
     <row r="4" spans="1:6" ht="26" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
@@ -3023,7 +3056,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BCCE9345-FC91-4D0C-9835-473AC28707EE}">
-  <dimension ref="B2:L12"/>
+  <dimension ref="B2:N29"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="16.08984375" bestFit="1" customWidth="1"/>
@@ -3420,8 +3453,549 @@
         <v>0</v>
       </c>
     </row>
+    <row r="17" spans="2:14" ht="29" x14ac:dyDescent="0.35">
+      <c r="B17" s="20"/>
+      <c r="C17" s="21" t="s">
+        <v>160</v>
+      </c>
+      <c r="D17" s="21" t="s">
+        <v>161</v>
+      </c>
+      <c r="E17" s="21" t="s">
+        <v>116</v>
+      </c>
+      <c r="F17" s="21" t="s">
+        <v>162</v>
+      </c>
+      <c r="G17" s="21" t="s">
+        <v>163</v>
+      </c>
+      <c r="H17" s="21" t="s">
+        <v>164</v>
+      </c>
+      <c r="I17" s="21" t="s">
+        <v>165</v>
+      </c>
+      <c r="J17" s="21" t="s">
+        <v>113</v>
+      </c>
+      <c r="K17" s="21" t="s">
+        <v>120</v>
+      </c>
+      <c r="L17" s="21" t="s">
+        <v>166</v>
+      </c>
+      <c r="M17" s="21" t="s">
+        <v>167</v>
+      </c>
+      <c r="N17" s="21" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="18" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B18" s="11" t="s">
+        <v>160</v>
+      </c>
+      <c r="C18" s="10">
+        <v>0</v>
+      </c>
+      <c r="D18" s="10">
+        <v>96</v>
+      </c>
+      <c r="E18" s="10">
+        <v>92</v>
+      </c>
+      <c r="F18" s="10">
+        <v>85</v>
+      </c>
+      <c r="G18" s="10">
+        <v>81</v>
+      </c>
+      <c r="H18" s="10">
+        <v>77</v>
+      </c>
+      <c r="I18" s="10">
+        <v>65</v>
+      </c>
+      <c r="J18" s="10">
+        <v>58</v>
+      </c>
+      <c r="K18" s="10">
+        <v>42</v>
+      </c>
+      <c r="L18" s="10">
+        <v>40</v>
+      </c>
+      <c r="M18" s="10">
+        <v>31</v>
+      </c>
+      <c r="N18" s="10">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="19" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B19" s="11" t="s">
+        <v>161</v>
+      </c>
+      <c r="C19" s="10">
+        <v>96</v>
+      </c>
+      <c r="D19" s="10">
+        <v>0</v>
+      </c>
+      <c r="E19" s="10">
+        <v>89</v>
+      </c>
+      <c r="F19" s="10">
+        <v>83</v>
+      </c>
+      <c r="G19" s="10">
+        <v>78</v>
+      </c>
+      <c r="H19" s="10">
+        <v>75</v>
+      </c>
+      <c r="I19" s="10">
+        <v>60</v>
+      </c>
+      <c r="J19" s="10">
+        <v>63</v>
+      </c>
+      <c r="K19" s="10">
+        <v>38</v>
+      </c>
+      <c r="L19" s="10">
+        <v>51</v>
+      </c>
+      <c r="M19" s="10">
+        <v>33</v>
+      </c>
+      <c r="N19" s="10">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="20" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B20" s="11" t="s">
+        <v>116</v>
+      </c>
+      <c r="C20" s="10">
+        <v>92</v>
+      </c>
+      <c r="D20" s="10">
+        <v>89</v>
+      </c>
+      <c r="E20" s="10">
+        <v>0</v>
+      </c>
+      <c r="F20" s="10">
+        <v>80</v>
+      </c>
+      <c r="G20" s="10">
+        <v>87</v>
+      </c>
+      <c r="H20" s="10">
+        <v>79</v>
+      </c>
+      <c r="I20" s="10">
+        <v>69</v>
+      </c>
+      <c r="J20" s="10">
+        <v>61</v>
+      </c>
+      <c r="K20" s="10">
+        <v>65</v>
+      </c>
+      <c r="L20" s="10">
+        <v>42</v>
+      </c>
+      <c r="M20" s="10">
+        <v>36</v>
+      </c>
+      <c r="N20" s="10">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="21" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B21" s="11" t="s">
+        <v>162</v>
+      </c>
+      <c r="C21" s="10">
+        <v>85</v>
+      </c>
+      <c r="D21" s="10">
+        <v>83</v>
+      </c>
+      <c r="E21" s="10">
+        <v>80</v>
+      </c>
+      <c r="F21" s="10">
+        <v>0</v>
+      </c>
+      <c r="G21" s="10">
+        <v>74</v>
+      </c>
+      <c r="H21" s="10">
+        <v>72</v>
+      </c>
+      <c r="I21" s="10">
+        <v>62</v>
+      </c>
+      <c r="J21" s="10">
+        <v>56</v>
+      </c>
+      <c r="K21" s="10">
+        <v>40</v>
+      </c>
+      <c r="L21" s="10">
+        <v>38</v>
+      </c>
+      <c r="M21" s="10">
+        <v>24</v>
+      </c>
+      <c r="N21" s="10">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="22" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B22" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="C22" s="10">
+        <v>81</v>
+      </c>
+      <c r="D22" s="10">
+        <v>78</v>
+      </c>
+      <c r="E22" s="10">
+        <v>87</v>
+      </c>
+      <c r="F22" s="10">
+        <v>74</v>
+      </c>
+      <c r="G22" s="10">
+        <v>0</v>
+      </c>
+      <c r="H22" s="10">
+        <v>83</v>
+      </c>
+      <c r="I22" s="10">
+        <v>71</v>
+      </c>
+      <c r="J22" s="10">
+        <v>53</v>
+      </c>
+      <c r="K22" s="10">
+        <v>49</v>
+      </c>
+      <c r="L22" s="10">
+        <v>35</v>
+      </c>
+      <c r="M22" s="10">
+        <v>47</v>
+      </c>
+      <c r="N22" s="10">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="23" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B23" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="C23" s="10">
+        <v>77</v>
+      </c>
+      <c r="D23" s="10">
+        <v>75</v>
+      </c>
+      <c r="E23" s="10">
+        <v>79</v>
+      </c>
+      <c r="F23" s="10">
+        <v>72</v>
+      </c>
+      <c r="G23" s="10">
+        <v>83</v>
+      </c>
+      <c r="H23" s="10">
+        <v>0</v>
+      </c>
+      <c r="I23" s="10">
+        <v>67</v>
+      </c>
+      <c r="J23" s="10">
+        <v>49</v>
+      </c>
+      <c r="K23" s="10">
+        <v>44</v>
+      </c>
+      <c r="L23" s="10">
+        <v>33</v>
+      </c>
+      <c r="M23" s="10">
+        <v>40</v>
+      </c>
+      <c r="N23" s="10">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="24" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B24" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="C24" s="10">
+        <v>65</v>
+      </c>
+      <c r="D24" s="10">
+        <v>60</v>
+      </c>
+      <c r="E24" s="10">
+        <v>69</v>
+      </c>
+      <c r="F24" s="10">
+        <v>62</v>
+      </c>
+      <c r="G24" s="10">
+        <v>71</v>
+      </c>
+      <c r="H24" s="10">
+        <v>67</v>
+      </c>
+      <c r="I24" s="10">
+        <v>0</v>
+      </c>
+      <c r="J24" s="10">
+        <v>44</v>
+      </c>
+      <c r="K24" s="10">
+        <v>47</v>
+      </c>
+      <c r="L24" s="10">
+        <v>27</v>
+      </c>
+      <c r="M24" s="10">
+        <v>35</v>
+      </c>
+      <c r="N24" s="10">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="25" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B25" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="C25" s="10">
+        <v>58</v>
+      </c>
+      <c r="D25" s="10">
+        <v>63</v>
+      </c>
+      <c r="E25" s="10">
+        <v>61</v>
+      </c>
+      <c r="F25" s="10">
+        <v>56</v>
+      </c>
+      <c r="G25" s="10">
+        <v>53</v>
+      </c>
+      <c r="H25" s="10">
+        <v>49</v>
+      </c>
+      <c r="I25" s="10">
+        <v>44</v>
+      </c>
+      <c r="J25" s="10">
+        <v>0</v>
+      </c>
+      <c r="K25" s="10">
+        <v>51</v>
+      </c>
+      <c r="L25" s="10">
+        <v>47</v>
+      </c>
+      <c r="M25" s="10">
+        <v>18</v>
+      </c>
+      <c r="N25" s="10">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="26" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B26" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="C26" s="10">
+        <v>42</v>
+      </c>
+      <c r="D26" s="10">
+        <v>38</v>
+      </c>
+      <c r="E26" s="10">
+        <v>65</v>
+      </c>
+      <c r="F26" s="10">
+        <v>40</v>
+      </c>
+      <c r="G26" s="10">
+        <v>49</v>
+      </c>
+      <c r="H26" s="10">
+        <v>44</v>
+      </c>
+      <c r="I26" s="10">
+        <v>47</v>
+      </c>
+      <c r="J26" s="10">
+        <v>51</v>
+      </c>
+      <c r="K26" s="10">
+        <v>0</v>
+      </c>
+      <c r="L26" s="10">
+        <v>31</v>
+      </c>
+      <c r="M26" s="10">
+        <v>15</v>
+      </c>
+      <c r="N26" s="10">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="27" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B27" s="11" t="s">
+        <v>166</v>
+      </c>
+      <c r="C27" s="10">
+        <v>40</v>
+      </c>
+      <c r="D27" s="10">
+        <v>51</v>
+      </c>
+      <c r="E27" s="10">
+        <v>42</v>
+      </c>
+      <c r="F27" s="10">
+        <v>38</v>
+      </c>
+      <c r="G27" s="10">
+        <v>35</v>
+      </c>
+      <c r="H27" s="10">
+        <v>33</v>
+      </c>
+      <c r="I27" s="10">
+        <v>27</v>
+      </c>
+      <c r="J27" s="10">
+        <v>47</v>
+      </c>
+      <c r="K27" s="10">
+        <v>31</v>
+      </c>
+      <c r="L27" s="10">
+        <v>0</v>
+      </c>
+      <c r="M27" s="10">
+        <v>13</v>
+      </c>
+      <c r="N27" s="10">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="28" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B28" s="11" t="s">
+        <v>167</v>
+      </c>
+      <c r="C28" s="10">
+        <v>31</v>
+      </c>
+      <c r="D28" s="10">
+        <v>33</v>
+      </c>
+      <c r="E28" s="10">
+        <v>36</v>
+      </c>
+      <c r="F28" s="10">
+        <v>24</v>
+      </c>
+      <c r="G28" s="10">
+        <v>47</v>
+      </c>
+      <c r="H28" s="10">
+        <v>40</v>
+      </c>
+      <c r="I28" s="10">
+        <v>35</v>
+      </c>
+      <c r="J28" s="10">
+        <v>18</v>
+      </c>
+      <c r="K28" s="10">
+        <v>15</v>
+      </c>
+      <c r="L28" s="10">
+        <v>13</v>
+      </c>
+      <c r="M28" s="10">
+        <v>0</v>
+      </c>
+      <c r="N28" s="10">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="29" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B29" s="11" t="s">
+        <v>168</v>
+      </c>
+      <c r="C29" s="10">
+        <v>35</v>
+      </c>
+      <c r="D29" s="10">
+        <v>29</v>
+      </c>
+      <c r="E29" s="10">
+        <v>44</v>
+      </c>
+      <c r="F29" s="10">
+        <v>31</v>
+      </c>
+      <c r="G29" s="10">
+        <v>56</v>
+      </c>
+      <c r="H29" s="10">
+        <v>51</v>
+      </c>
+      <c r="I29" s="10">
+        <v>49</v>
+      </c>
+      <c r="J29" s="10">
+        <v>22</v>
+      </c>
+      <c r="K29" s="10">
+        <v>27</v>
+      </c>
+      <c r="L29" s="10">
+        <v>11</v>
+      </c>
+      <c r="M29" s="10">
+        <v>42</v>
+      </c>
+      <c r="N29" s="10">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="C3:L12">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C18:N29">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -5931,10 +6505,10 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="2" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="15" t="s">
         <v>151</v>
       </c>
-      <c r="C2" s="19" t="s">
+      <c r="C2" s="15" t="s">
         <v>152</v>
       </c>
     </row>
@@ -5947,10 +6521,10 @@
       </c>
     </row>
     <row r="4" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="15" t="s">
         <v>151</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="15" t="s">
         <v>153</v>
       </c>
     </row>
@@ -5963,10 +6537,10 @@
       </c>
     </row>
     <row r="6" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="15" t="s">
         <v>156</v>
       </c>
-      <c r="C6" s="19" t="s">
+      <c r="C6" s="15" t="s">
         <v>157</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added metrcs from claude and chatGPT
</commit_message>
<xml_diff>
--- a/ms_teams_copilot_client_answers.xlsx
+++ b/ms_teams_copilot_client_answers.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MohitVerma\Desktop\git\translation\SaS-to-python\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BAE94EB-60A4-423B-B914-5A266A83621C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4553A32C-6C30-4071-A597-925901DCB89B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="300" windowWidth="19420" windowHeight="10420" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Quick Summary" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="176">
   <si>
     <t>Quick summary for the client</t>
   </si>
@@ -691,6 +691,27 @@
   </si>
   <si>
     <t>PNC Bank</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Synchrony </t>
+  </si>
+  <si>
+    <t>Gemini</t>
+  </si>
+  <si>
+    <t>Claude</t>
+  </si>
+  <si>
+    <t>JP Morgan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PNC Bank </t>
+  </si>
+  <si>
+    <t>GoldmanSachs</t>
+  </si>
+  <si>
+    <t>ChatGPT</t>
   </si>
 </sst>
 </file>
@@ -877,6 +898,12 @@
       <alignment vertical="center" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -886,12 +913,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2433,22 +2454,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
     </row>
     <row r="2" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
     </row>
     <row r="4" spans="1:5" ht="26" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
@@ -2646,40 +2667,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
     </row>
     <row r="2" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="21" t="s">
         <v>38</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
-      <c r="H2" s="17"/>
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
+      <c r="H2" s="19"/>
     </row>
     <row r="3" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="16" t="s">
+      <c r="A3" s="18" t="s">
         <v>39</v>
       </c>
-      <c r="B3" s="17"/>
-      <c r="C3" s="17"/>
-      <c r="D3" s="17"/>
-      <c r="E3" s="17"/>
-      <c r="F3" s="17"/>
-      <c r="G3" s="17"/>
-      <c r="H3" s="17"/>
+      <c r="B3" s="19"/>
+      <c r="C3" s="19"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="19"/>
+      <c r="G3" s="19"/>
+      <c r="H3" s="19"/>
     </row>
     <row r="4" spans="1:8" ht="26" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
@@ -2965,24 +2986,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="20" t="s">
         <v>94</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
     </row>
     <row r="2" spans="1:6" ht="42" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
     </row>
     <row r="4" spans="1:6" ht="26" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
@@ -3056,7 +3077,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BCCE9345-FC91-4D0C-9835-473AC28707EE}">
-  <dimension ref="B2:N29"/>
+  <dimension ref="B1:AP30"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="16.08984375" bestFit="1" customWidth="1"/>
@@ -3068,924 +3089,2709 @@
     <col min="14" max="14" width="11.81640625" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="13.1796875" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="12.6328125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="14.54296875" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="15.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B2" s="10"/>
-      <c r="C2" s="11" t="s">
+    <row r="1" spans="2:40" x14ac:dyDescent="0.35">
+      <c r="B1" t="s">
+        <v>170</v>
+      </c>
+      <c r="P1" t="s">
+        <v>171</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="3" spans="2:40" x14ac:dyDescent="0.35">
+      <c r="B3" s="10"/>
+      <c r="C3" s="11" t="s">
         <v>112</v>
       </c>
-      <c r="D2" s="11" t="s">
+      <c r="D3" s="11" t="s">
         <v>113</v>
       </c>
-      <c r="E2" s="11" t="s">
+      <c r="E3" s="11" t="s">
         <v>114</v>
       </c>
-      <c r="F2" s="11" t="s">
+      <c r="F3" s="11" t="s">
         <v>115</v>
       </c>
-      <c r="G2" s="11" t="s">
+      <c r="G3" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="H2" s="11" t="s">
+      <c r="H3" s="11" t="s">
         <v>117</v>
       </c>
-      <c r="I2" s="11" t="s">
+      <c r="I3" s="11" t="s">
         <v>118</v>
       </c>
-      <c r="J2" s="11" t="s">
+      <c r="J3" s="11" t="s">
         <v>121</v>
       </c>
-      <c r="K2" s="11" t="s">
+      <c r="K3" s="11" t="s">
         <v>119</v>
       </c>
-      <c r="L2" s="11" t="s">
+      <c r="L3" s="11" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="3" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B3" s="11" t="s">
+      <c r="P3" s="10"/>
+      <c r="Q3" s="11" t="s">
         <v>112</v>
       </c>
-      <c r="C3" s="10">
+      <c r="R3" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="S3" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="T3" s="11" t="s">
+        <v>115</v>
+      </c>
+      <c r="U3" s="11" t="s">
+        <v>116</v>
+      </c>
+      <c r="V3" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="W3" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="X3" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="Y3" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="Z3" s="11" t="s">
+        <v>169</v>
+      </c>
+      <c r="AD3" s="10"/>
+      <c r="AE3" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="AF3" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="AG3" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="AH3" s="11" t="s">
+        <v>115</v>
+      </c>
+      <c r="AI3" s="11" t="s">
+        <v>116</v>
+      </c>
+      <c r="AJ3" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="AK3" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="AL3" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="AM3" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="AN3" s="11" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="4" spans="2:40" x14ac:dyDescent="0.35">
+      <c r="B4" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="C4" s="10">
         <v>0</v>
       </c>
-      <c r="D3" s="10">
+      <c r="D4" s="10">
         <v>38</v>
       </c>
-      <c r="E3" s="10">
+      <c r="E4" s="10">
         <v>58</v>
       </c>
-      <c r="F3" s="10">
+      <c r="F4" s="10">
         <v>73</v>
       </c>
-      <c r="G3" s="10">
+      <c r="G4" s="10">
         <v>80</v>
       </c>
-      <c r="H3" s="10">
+      <c r="H4" s="10">
         <v>67</v>
       </c>
-      <c r="I3" s="10">
+      <c r="I4" s="10">
         <v>60</v>
       </c>
-      <c r="J3" s="10">
+      <c r="J4" s="10">
         <v>62</v>
       </c>
-      <c r="K3" s="10">
+      <c r="K4" s="10">
         <v>49</v>
       </c>
-      <c r="L3" s="10">
+      <c r="L4" s="10">
         <v>31</v>
       </c>
-    </row>
-    <row r="4" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B4" s="11" t="s">
+      <c r="P4" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="Q4" s="10">
+        <v>0</v>
+      </c>
+      <c r="R4" s="10">
+        <v>23</v>
+      </c>
+      <c r="S4" s="10">
+        <v>93</v>
+      </c>
+      <c r="T4" s="10">
+        <v>86</v>
+      </c>
+      <c r="U4" s="10">
+        <v>73</v>
+      </c>
+      <c r="V4" s="10">
+        <v>75</v>
+      </c>
+      <c r="W4" s="10">
+        <v>50</v>
+      </c>
+      <c r="X4" s="10">
+        <v>91</v>
+      </c>
+      <c r="Y4" s="10">
+        <v>48</v>
+      </c>
+      <c r="Z4" s="10">
+        <v>21</v>
+      </c>
+      <c r="AD4" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="AE4" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF4" s="10">
+        <v>18</v>
+      </c>
+      <c r="AG4" s="10">
+        <v>34</v>
+      </c>
+      <c r="AH4" s="10">
+        <v>62</v>
+      </c>
+      <c r="AI4" s="10">
+        <v>88</v>
+      </c>
+      <c r="AJ4" s="10">
+        <v>76</v>
+      </c>
+      <c r="AK4" s="10">
+        <v>71</v>
+      </c>
+      <c r="AL4" s="10">
+        <v>55</v>
+      </c>
+      <c r="AM4" s="10">
+        <v>22</v>
+      </c>
+      <c r="AN4" s="10">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="5" spans="2:40" x14ac:dyDescent="0.35">
+      <c r="B5" s="11" t="s">
         <v>113</v>
       </c>
-      <c r="C4" s="10">
+      <c r="C5" s="10">
         <v>38</v>
       </c>
-      <c r="D4" s="10">
+      <c r="D5" s="10">
         <v>0</v>
       </c>
-      <c r="E4" s="10">
+      <c r="E5" s="10">
         <v>40</v>
       </c>
-      <c r="F4" s="10">
+      <c r="F5" s="10">
         <v>42</v>
       </c>
-      <c r="G4" s="10">
+      <c r="G5" s="10">
         <v>56</v>
       </c>
-      <c r="H4" s="10">
+      <c r="H5" s="10">
         <v>53</v>
       </c>
-      <c r="I4" s="10">
+      <c r="I5" s="10">
         <v>64</v>
       </c>
-      <c r="J4" s="10">
+      <c r="J5" s="10">
         <v>36</v>
       </c>
-      <c r="K4" s="10">
+      <c r="K5" s="10">
         <v>22</v>
       </c>
-      <c r="L4" s="10">
+      <c r="L5" s="10">
         <v>27</v>
       </c>
-    </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B5" s="11" t="s">
+      <c r="P5" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="Q5" s="10">
+        <v>23</v>
+      </c>
+      <c r="R5" s="10">
+        <v>0</v>
+      </c>
+      <c r="S5" s="10">
+        <v>28</v>
+      </c>
+      <c r="T5" s="10">
+        <v>35</v>
+      </c>
+      <c r="U5" s="10">
+        <v>44</v>
+      </c>
+      <c r="V5" s="10">
+        <v>41</v>
+      </c>
+      <c r="W5" s="10">
+        <v>39</v>
+      </c>
+      <c r="X5" s="10">
+        <v>30</v>
+      </c>
+      <c r="Y5" s="10">
+        <v>1</v>
+      </c>
+      <c r="Z5" s="10">
+        <v>5</v>
+      </c>
+      <c r="AD5" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="AE5" s="10">
+        <v>18</v>
+      </c>
+      <c r="AF5" s="10">
+        <v>0</v>
+      </c>
+      <c r="AG5" s="10">
+        <v>12</v>
+      </c>
+      <c r="AH5" s="10">
+        <v>29</v>
+      </c>
+      <c r="AI5" s="10">
+        <v>74</v>
+      </c>
+      <c r="AJ5" s="10">
+        <v>58</v>
+      </c>
+      <c r="AK5" s="10">
+        <v>66</v>
+      </c>
+      <c r="AL5" s="10">
+        <v>24</v>
+      </c>
+      <c r="AM5" s="10">
+        <v>1</v>
+      </c>
+      <c r="AN5" s="10">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" spans="2:40" x14ac:dyDescent="0.35">
+      <c r="B6" s="11" t="s">
         <v>114</v>
       </c>
-      <c r="C5" s="10">
+      <c r="C6" s="10">
         <v>58</v>
       </c>
-      <c r="D5" s="10">
+      <c r="D6" s="10">
         <v>40</v>
       </c>
-      <c r="E5" s="10">
+      <c r="E6" s="10">
         <v>0</v>
       </c>
-      <c r="F5" s="10">
+      <c r="F6" s="10">
         <v>69</v>
       </c>
-      <c r="G5" s="10">
+      <c r="G6" s="10">
         <v>51</v>
       </c>
-      <c r="H5" s="10">
+      <c r="H6" s="10">
         <v>47</v>
       </c>
-      <c r="I5" s="10">
+      <c r="I6" s="10">
         <v>44</v>
       </c>
-      <c r="J5" s="10">
+      <c r="J6" s="10">
         <v>82</v>
       </c>
-      <c r="K5" s="10">
+      <c r="K6" s="10">
         <v>53</v>
       </c>
-      <c r="L5" s="10">
+      <c r="L6" s="10">
         <v>33</v>
       </c>
-    </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B6" s="11" t="s">
+      <c r="P6" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="Q6" s="10">
+        <v>93</v>
+      </c>
+      <c r="R6" s="10">
+        <v>28</v>
+      </c>
+      <c r="S6" s="10">
+        <v>0</v>
+      </c>
+      <c r="T6" s="10">
+        <v>82</v>
+      </c>
+      <c r="U6" s="10">
+        <v>57</v>
+      </c>
+      <c r="V6" s="10">
+        <v>64</v>
+      </c>
+      <c r="W6" s="10">
+        <v>59</v>
+      </c>
+      <c r="X6" s="10">
+        <v>89</v>
+      </c>
+      <c r="Y6" s="10">
+        <v>26</v>
+      </c>
+      <c r="Z6" s="10">
+        <v>8</v>
+      </c>
+      <c r="AD6" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="AE6" s="10">
+        <v>34</v>
+      </c>
+      <c r="AF6" s="10">
+        <v>12</v>
+      </c>
+      <c r="AG6" s="10">
+        <v>0</v>
+      </c>
+      <c r="AH6" s="10">
+        <v>44</v>
+      </c>
+      <c r="AI6" s="10">
+        <v>79</v>
+      </c>
+      <c r="AJ6" s="10">
+        <v>63</v>
+      </c>
+      <c r="AK6" s="10">
+        <v>57</v>
+      </c>
+      <c r="AL6" s="10">
+        <v>41</v>
+      </c>
+      <c r="AM6" s="10">
+        <v>15</v>
+      </c>
+      <c r="AN6" s="10">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7" spans="2:40" x14ac:dyDescent="0.35">
+      <c r="B7" s="11" t="s">
         <v>115</v>
       </c>
-      <c r="C6" s="10">
+      <c r="C7" s="10">
         <v>73</v>
       </c>
-      <c r="D6" s="10">
+      <c r="D7" s="10">
         <v>42</v>
       </c>
-      <c r="E6" s="10">
+      <c r="E7" s="10">
         <v>69</v>
       </c>
-      <c r="F6" s="10">
+      <c r="F7" s="10">
         <v>0</v>
       </c>
-      <c r="G6" s="10">
+      <c r="G7" s="10">
         <v>84</v>
       </c>
-      <c r="H6" s="10">
+      <c r="H7" s="10">
         <v>78</v>
       </c>
-      <c r="I6" s="10">
+      <c r="I7" s="10">
         <v>71</v>
       </c>
-      <c r="J6" s="10">
+      <c r="J7" s="10">
         <v>60</v>
       </c>
-      <c r="K6" s="10">
+      <c r="K7" s="10">
         <v>47</v>
       </c>
-      <c r="L6" s="10">
+      <c r="L7" s="10">
         <v>36</v>
       </c>
-    </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B7" s="11" t="s">
+      <c r="P7" s="11" t="s">
+        <v>115</v>
+      </c>
+      <c r="Q7" s="10">
+        <v>86</v>
+      </c>
+      <c r="R7" s="10">
+        <v>35</v>
+      </c>
+      <c r="S7" s="10">
+        <v>82</v>
+      </c>
+      <c r="T7" s="10">
+        <v>0</v>
+      </c>
+      <c r="U7" s="10">
+        <v>71</v>
+      </c>
+      <c r="V7" s="10">
+        <v>66</v>
+      </c>
+      <c r="W7" s="10">
+        <v>62</v>
+      </c>
+      <c r="X7" s="10">
+        <v>84</v>
+      </c>
+      <c r="Y7" s="10">
+        <v>19</v>
+      </c>
+      <c r="Z7" s="10">
+        <v>37</v>
+      </c>
+      <c r="AD7" s="11" t="s">
+        <v>115</v>
+      </c>
+      <c r="AE7" s="10">
+        <v>62</v>
+      </c>
+      <c r="AF7" s="10">
+        <v>29</v>
+      </c>
+      <c r="AG7" s="10">
+        <v>44</v>
+      </c>
+      <c r="AH7" s="10">
+        <v>0</v>
+      </c>
+      <c r="AI7" s="10">
+        <v>95</v>
+      </c>
+      <c r="AJ7" s="10">
+        <v>82</v>
+      </c>
+      <c r="AK7" s="10">
+        <v>77</v>
+      </c>
+      <c r="AL7" s="10">
+        <v>69</v>
+      </c>
+      <c r="AM7" s="10">
+        <v>27</v>
+      </c>
+      <c r="AN7" s="10">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="8" spans="2:40" x14ac:dyDescent="0.35">
+      <c r="B8" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="C7" s="10">
+      <c r="C8" s="10">
         <v>80</v>
       </c>
-      <c r="D7" s="10">
+      <c r="D8" s="10">
         <v>56</v>
       </c>
-      <c r="E7" s="10">
+      <c r="E8" s="10">
         <v>51</v>
       </c>
-      <c r="F7" s="10">
+      <c r="F8" s="10">
         <v>84</v>
       </c>
-      <c r="G7" s="10">
+      <c r="G8" s="10">
         <v>0</v>
       </c>
-      <c r="H7" s="10">
+      <c r="H8" s="10">
         <v>98</v>
       </c>
-      <c r="I7" s="10">
+      <c r="I8" s="10">
         <v>96</v>
       </c>
-      <c r="J7" s="10">
+      <c r="J8" s="10">
         <v>76</v>
       </c>
-      <c r="K7" s="10">
+      <c r="K8" s="10">
         <v>42</v>
       </c>
-      <c r="L7" s="10">
+      <c r="L8" s="10">
         <v>62</v>
       </c>
-    </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B8" s="11" t="s">
+      <c r="P8" s="11" t="s">
+        <v>116</v>
+      </c>
+      <c r="Q8" s="10">
+        <v>73</v>
+      </c>
+      <c r="R8" s="10">
+        <v>44</v>
+      </c>
+      <c r="S8" s="10">
+        <v>57</v>
+      </c>
+      <c r="T8" s="10">
+        <v>71</v>
+      </c>
+      <c r="U8" s="10">
+        <v>0</v>
+      </c>
+      <c r="V8" s="10">
+        <v>100</v>
+      </c>
+      <c r="W8" s="10">
+        <v>98</v>
+      </c>
+      <c r="X8" s="10">
+        <v>77</v>
+      </c>
+      <c r="Y8" s="10">
+        <v>17</v>
+      </c>
+      <c r="Z8" s="10">
+        <v>53</v>
+      </c>
+      <c r="AD8" s="11" t="s">
+        <v>116</v>
+      </c>
+      <c r="AE8" s="10">
+        <v>88</v>
+      </c>
+      <c r="AF8" s="10">
+        <v>74</v>
+      </c>
+      <c r="AG8" s="10">
+        <v>79</v>
+      </c>
+      <c r="AH8" s="10">
+        <v>95</v>
+      </c>
+      <c r="AI8" s="10">
+        <v>0</v>
+      </c>
+      <c r="AJ8" s="10">
+        <v>100</v>
+      </c>
+      <c r="AK8" s="10">
+        <v>97</v>
+      </c>
+      <c r="AL8" s="10">
+        <v>84</v>
+      </c>
+      <c r="AM8" s="10">
+        <v>49</v>
+      </c>
+      <c r="AN8" s="10">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="9" spans="2:40" x14ac:dyDescent="0.35">
+      <c r="B9" s="11" t="s">
         <v>117</v>
       </c>
-      <c r="C8" s="10">
+      <c r="C9" s="10">
         <v>67</v>
       </c>
-      <c r="D8" s="10">
+      <c r="D9" s="10">
         <v>53</v>
       </c>
-      <c r="E8" s="10">
+      <c r="E9" s="10">
         <v>47</v>
       </c>
-      <c r="F8" s="10">
+      <c r="F9" s="10">
         <v>78</v>
       </c>
-      <c r="G8" s="10">
+      <c r="G9" s="10">
         <v>98</v>
       </c>
-      <c r="H8" s="10">
+      <c r="H9" s="10">
         <v>0</v>
       </c>
-      <c r="I8" s="10">
+      <c r="I9" s="10">
         <v>93</v>
       </c>
-      <c r="J8" s="10">
+      <c r="J9" s="10">
         <v>56</v>
       </c>
-      <c r="K8" s="10">
+      <c r="K9" s="10">
         <v>31</v>
       </c>
-      <c r="L8" s="10">
+      <c r="L9" s="10">
         <v>71</v>
       </c>
-    </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B9" s="11" t="s">
+      <c r="P9" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="Q9" s="10">
+        <v>75</v>
+      </c>
+      <c r="R9" s="10">
+        <v>41</v>
+      </c>
+      <c r="S9" s="10">
+        <v>64</v>
+      </c>
+      <c r="T9" s="10">
+        <v>66</v>
+      </c>
+      <c r="U9" s="10">
+        <v>100</v>
+      </c>
+      <c r="V9" s="10">
+        <v>0</v>
+      </c>
+      <c r="W9" s="10">
+        <v>95</v>
+      </c>
+      <c r="X9" s="10">
+        <v>80</v>
+      </c>
+      <c r="Y9" s="10">
+        <v>14</v>
+      </c>
+      <c r="Z9" s="10">
+        <v>55</v>
+      </c>
+      <c r="AD9" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="AE9" s="10">
+        <v>76</v>
+      </c>
+      <c r="AF9" s="10">
+        <v>58</v>
+      </c>
+      <c r="AG9" s="10">
+        <v>63</v>
+      </c>
+      <c r="AH9" s="10">
+        <v>82</v>
+      </c>
+      <c r="AI9" s="10">
+        <v>100</v>
+      </c>
+      <c r="AJ9" s="10">
+        <v>0</v>
+      </c>
+      <c r="AK9" s="10">
+        <v>92</v>
+      </c>
+      <c r="AL9" s="10">
+        <v>73</v>
+      </c>
+      <c r="AM9" s="10">
+        <v>39</v>
+      </c>
+      <c r="AN9" s="10">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="10" spans="2:40" x14ac:dyDescent="0.35">
+      <c r="B10" s="11" t="s">
         <v>118</v>
       </c>
-      <c r="C9" s="10">
+      <c r="C10" s="10">
         <v>60</v>
       </c>
-      <c r="D9" s="10">
+      <c r="D10" s="10">
         <v>64</v>
       </c>
-      <c r="E9" s="10">
+      <c r="E10" s="10">
         <v>44</v>
       </c>
-      <c r="F9" s="10">
+      <c r="F10" s="10">
         <v>71</v>
       </c>
-      <c r="G9" s="10">
+      <c r="G10" s="10">
         <v>96</v>
       </c>
-      <c r="H9" s="10">
+      <c r="H10" s="10">
         <v>93</v>
       </c>
-      <c r="I9" s="10">
+      <c r="I10" s="10">
         <v>0</v>
       </c>
-      <c r="J9" s="10">
+      <c r="J10" s="10">
         <v>64</v>
       </c>
-      <c r="K9" s="10">
+      <c r="K10" s="10">
         <v>24</v>
       </c>
-      <c r="L9" s="10">
+      <c r="L10" s="10">
         <v>67</v>
       </c>
-    </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B10" s="11" t="s">
+      <c r="P10" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="Q10" s="10">
+        <v>50</v>
+      </c>
+      <c r="R10" s="10">
+        <v>39</v>
+      </c>
+      <c r="S10" s="10">
+        <v>59</v>
+      </c>
+      <c r="T10" s="10">
+        <v>62</v>
+      </c>
+      <c r="U10" s="10">
+        <v>98</v>
+      </c>
+      <c r="V10" s="10">
+        <v>95</v>
+      </c>
+      <c r="W10" s="10">
+        <v>0</v>
+      </c>
+      <c r="X10" s="10">
+        <v>68</v>
+      </c>
+      <c r="Y10" s="10">
+        <v>10</v>
+      </c>
+      <c r="Z10" s="10">
+        <v>46</v>
+      </c>
+      <c r="AD10" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="AE10" s="10">
+        <v>71</v>
+      </c>
+      <c r="AF10" s="10">
+        <v>66</v>
+      </c>
+      <c r="AG10" s="10">
+        <v>57</v>
+      </c>
+      <c r="AH10" s="10">
+        <v>77</v>
+      </c>
+      <c r="AI10" s="10">
+        <v>97</v>
+      </c>
+      <c r="AJ10" s="10">
+        <v>92</v>
+      </c>
+      <c r="AK10" s="10">
+        <v>0</v>
+      </c>
+      <c r="AL10" s="10">
+        <v>68</v>
+      </c>
+      <c r="AM10" s="10">
+        <v>33</v>
+      </c>
+      <c r="AN10" s="10">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="11" spans="2:40" x14ac:dyDescent="0.35">
+      <c r="B11" s="11" t="s">
         <v>121</v>
       </c>
-      <c r="C10" s="10">
+      <c r="C11" s="10">
         <v>62</v>
       </c>
-      <c r="D10" s="10">
+      <c r="D11" s="10">
         <v>36</v>
       </c>
-      <c r="E10" s="10">
+      <c r="E11" s="10">
         <v>82</v>
       </c>
-      <c r="F10" s="10">
+      <c r="F11" s="10">
         <v>60</v>
       </c>
-      <c r="G10" s="10">
+      <c r="G11" s="10">
         <v>76</v>
       </c>
-      <c r="H10" s="10">
+      <c r="H11" s="10">
         <v>56</v>
       </c>
-      <c r="I10" s="10">
+      <c r="I11" s="10">
         <v>64</v>
       </c>
-      <c r="J10" s="10">
+      <c r="J11" s="10">
         <v>0</v>
       </c>
-      <c r="K10" s="10">
+      <c r="K11" s="10">
         <v>40</v>
       </c>
-      <c r="L10" s="10">
+      <c r="L11" s="10">
         <v>29</v>
       </c>
-    </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B11" s="11" t="s">
+      <c r="P11" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="Q11" s="10">
+        <v>91</v>
+      </c>
+      <c r="R11" s="10">
+        <v>30</v>
+      </c>
+      <c r="S11" s="10">
+        <v>89</v>
+      </c>
+      <c r="T11" s="10">
+        <v>84</v>
+      </c>
+      <c r="U11" s="10">
+        <v>77</v>
+      </c>
+      <c r="V11" s="10">
+        <v>80</v>
+      </c>
+      <c r="W11" s="10">
+        <v>68</v>
+      </c>
+      <c r="X11" s="10">
+        <v>0</v>
+      </c>
+      <c r="Y11" s="10">
+        <v>12</v>
+      </c>
+      <c r="Z11" s="10">
+        <v>32</v>
+      </c>
+      <c r="AD11" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="AE11" s="10">
+        <v>55</v>
+      </c>
+      <c r="AF11" s="10">
+        <v>24</v>
+      </c>
+      <c r="AG11" s="10">
+        <v>41</v>
+      </c>
+      <c r="AH11" s="10">
+        <v>69</v>
+      </c>
+      <c r="AI11" s="10">
+        <v>84</v>
+      </c>
+      <c r="AJ11" s="10">
+        <v>73</v>
+      </c>
+      <c r="AK11" s="10">
+        <v>68</v>
+      </c>
+      <c r="AL11" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM11" s="10">
+        <v>20</v>
+      </c>
+      <c r="AN11" s="10">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="12" spans="2:40" x14ac:dyDescent="0.35">
+      <c r="B12" s="11" t="s">
         <v>119</v>
       </c>
-      <c r="C11" s="10">
+      <c r="C12" s="10">
         <v>49</v>
       </c>
-      <c r="D11" s="10">
+      <c r="D12" s="10">
         <v>22</v>
       </c>
-      <c r="E11" s="10">
+      <c r="E12" s="10">
         <v>53</v>
       </c>
-      <c r="F11" s="10">
+      <c r="F12" s="10">
         <v>47</v>
       </c>
-      <c r="G11" s="10">
+      <c r="G12" s="10">
         <v>42</v>
       </c>
-      <c r="H11" s="10">
+      <c r="H12" s="10">
         <v>31</v>
       </c>
-      <c r="I11" s="10">
+      <c r="I12" s="10">
         <v>24</v>
       </c>
-      <c r="J11" s="10">
+      <c r="J12" s="10">
         <v>40</v>
       </c>
-      <c r="K11" s="10">
+      <c r="K12" s="10">
         <v>0</v>
       </c>
-      <c r="L11" s="10">
+      <c r="L12" s="10">
         <v>18</v>
       </c>
-    </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B12" s="11" t="s">
+      <c r="P12" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="Q12" s="10">
+        <v>48</v>
+      </c>
+      <c r="R12" s="10">
+        <v>1</v>
+      </c>
+      <c r="S12" s="10">
+        <v>26</v>
+      </c>
+      <c r="T12" s="10">
+        <v>19</v>
+      </c>
+      <c r="U12" s="10">
+        <v>17</v>
+      </c>
+      <c r="V12" s="10">
+        <v>14</v>
+      </c>
+      <c r="W12" s="10">
+        <v>10</v>
+      </c>
+      <c r="X12" s="10">
+        <v>12</v>
+      </c>
+      <c r="Y12" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z12" s="10">
+        <v>3</v>
+      </c>
+      <c r="AD12" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="AE12" s="10">
+        <v>22</v>
+      </c>
+      <c r="AF12" s="10">
+        <v>1</v>
+      </c>
+      <c r="AG12" s="10">
+        <v>15</v>
+      </c>
+      <c r="AH12" s="10">
+        <v>27</v>
+      </c>
+      <c r="AI12" s="10">
+        <v>49</v>
+      </c>
+      <c r="AJ12" s="10">
+        <v>39</v>
+      </c>
+      <c r="AK12" s="10">
+        <v>33</v>
+      </c>
+      <c r="AL12" s="10">
+        <v>20</v>
+      </c>
+      <c r="AM12" s="10">
+        <v>0</v>
+      </c>
+      <c r="AN12" s="10">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13" spans="2:40" x14ac:dyDescent="0.35">
+      <c r="B13" s="11" t="s">
         <v>120</v>
       </c>
-      <c r="C12" s="10">
+      <c r="C13" s="10">
         <v>31</v>
       </c>
-      <c r="D12" s="10">
+      <c r="D13" s="10">
         <v>27</v>
       </c>
-      <c r="E12" s="10">
+      <c r="E13" s="10">
         <v>33</v>
       </c>
-      <c r="F12" s="10">
+      <c r="F13" s="10">
         <v>36</v>
       </c>
-      <c r="G12" s="10">
+      <c r="G13" s="10">
         <v>62</v>
       </c>
-      <c r="H12" s="10">
+      <c r="H13" s="10">
         <v>71</v>
       </c>
-      <c r="I12" s="10">
+      <c r="I13" s="10">
         <v>67</v>
       </c>
-      <c r="J12" s="10">
+      <c r="J13" s="10">
         <v>29</v>
       </c>
-      <c r="K12" s="10">
+      <c r="K13" s="10">
         <v>18</v>
       </c>
-      <c r="L12" s="10">
+      <c r="L13" s="10">
         <v>0</v>
       </c>
-    </row>
-    <row r="17" spans="2:14" ht="29" x14ac:dyDescent="0.35">
-      <c r="B17" s="20"/>
-      <c r="C17" s="21" t="s">
+      <c r="P13" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="Q13" s="10">
+        <v>21</v>
+      </c>
+      <c r="R13" s="10">
+        <v>5</v>
+      </c>
+      <c r="S13" s="10">
+        <v>8</v>
+      </c>
+      <c r="T13" s="10">
+        <v>37</v>
+      </c>
+      <c r="U13" s="10">
+        <v>53</v>
+      </c>
+      <c r="V13" s="10">
+        <v>55</v>
+      </c>
+      <c r="W13" s="10">
+        <v>46</v>
+      </c>
+      <c r="X13" s="10">
+        <v>32</v>
+      </c>
+      <c r="Y13" s="10">
+        <v>3</v>
+      </c>
+      <c r="Z13" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD13" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="AE13" s="10">
+        <v>47</v>
+      </c>
+      <c r="AF13" s="10">
+        <v>31</v>
+      </c>
+      <c r="AG13" s="10">
+        <v>36</v>
+      </c>
+      <c r="AH13" s="10">
+        <v>53</v>
+      </c>
+      <c r="AI13" s="10">
+        <v>86</v>
+      </c>
+      <c r="AJ13" s="10">
+        <v>81</v>
+      </c>
+      <c r="AK13" s="10">
+        <v>89</v>
+      </c>
+      <c r="AL13" s="10">
+        <v>51</v>
+      </c>
+      <c r="AM13" s="10">
+        <v>26</v>
+      </c>
+      <c r="AN13" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="2:42" ht="29" x14ac:dyDescent="0.35">
+      <c r="B18" s="16"/>
+      <c r="C18" s="17" t="s">
         <v>160</v>
       </c>
-      <c r="D17" s="21" t="s">
+      <c r="D18" s="17" t="s">
         <v>161</v>
       </c>
-      <c r="E17" s="21" t="s">
+      <c r="E18" s="17" t="s">
         <v>116</v>
       </c>
-      <c r="F17" s="21" t="s">
+      <c r="F18" s="17" t="s">
         <v>162</v>
       </c>
-      <c r="G17" s="21" t="s">
+      <c r="G18" s="17" t="s">
         <v>163</v>
       </c>
-      <c r="H17" s="21" t="s">
+      <c r="H18" s="17" t="s">
         <v>164</v>
       </c>
-      <c r="I17" s="21" t="s">
+      <c r="I18" s="17" t="s">
         <v>165</v>
       </c>
-      <c r="J17" s="21" t="s">
+      <c r="J18" s="17" t="s">
         <v>113</v>
       </c>
-      <c r="K17" s="21" t="s">
+      <c r="K18" s="17" t="s">
         <v>120</v>
       </c>
-      <c r="L17" s="21" t="s">
+      <c r="L18" s="17" t="s">
         <v>166</v>
       </c>
-      <c r="M17" s="21" t="s">
+      <c r="M18" s="17" t="s">
         <v>167</v>
       </c>
-      <c r="N17" s="21" t="s">
+      <c r="N18" s="17" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="18" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B18" s="11" t="s">
+      <c r="P18" s="16"/>
+      <c r="Q18" s="17" t="s">
+        <v>172</v>
+      </c>
+      <c r="R18" s="17" t="s">
+        <v>161</v>
+      </c>
+      <c r="S18" s="17" t="s">
+        <v>116</v>
+      </c>
+      <c r="T18" s="17" t="s">
+        <v>162</v>
+      </c>
+      <c r="U18" s="17" t="s">
+        <v>163</v>
+      </c>
+      <c r="V18" s="17" t="s">
+        <v>164</v>
+      </c>
+      <c r="W18" s="17" t="s">
+        <v>165</v>
+      </c>
+      <c r="X18" s="17" t="s">
+        <v>113</v>
+      </c>
+      <c r="Y18" s="17" t="s">
+        <v>120</v>
+      </c>
+      <c r="Z18" s="17" t="s">
+        <v>166</v>
+      </c>
+      <c r="AA18" s="17" t="s">
+        <v>167</v>
+      </c>
+      <c r="AB18" s="17" t="s">
+        <v>173</v>
+      </c>
+      <c r="AD18" s="16"/>
+      <c r="AE18" s="17" t="s">
         <v>160</v>
       </c>
-      <c r="C18" s="10">
+      <c r="AF18" s="17" t="s">
+        <v>161</v>
+      </c>
+      <c r="AG18" s="17" t="s">
+        <v>116</v>
+      </c>
+      <c r="AH18" s="17" t="s">
+        <v>162</v>
+      </c>
+      <c r="AI18" s="17" t="s">
+        <v>163</v>
+      </c>
+      <c r="AJ18" s="17" t="s">
+        <v>164</v>
+      </c>
+      <c r="AK18" s="17" t="s">
+        <v>165</v>
+      </c>
+      <c r="AL18" s="17" t="s">
+        <v>113</v>
+      </c>
+      <c r="AM18" s="17" t="s">
+        <v>120</v>
+      </c>
+      <c r="AN18" s="17" t="s">
+        <v>174</v>
+      </c>
+      <c r="AO18" s="17" t="s">
+        <v>167</v>
+      </c>
+      <c r="AP18" s="17" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="19" spans="2:42" x14ac:dyDescent="0.35">
+      <c r="B19" s="11" t="s">
+        <v>160</v>
+      </c>
+      <c r="C19" s="10">
         <v>0</v>
       </c>
-      <c r="D18" s="10">
+      <c r="D19" s="10">
         <v>96</v>
       </c>
-      <c r="E18" s="10">
+      <c r="E19" s="10">
         <v>92</v>
       </c>
-      <c r="F18" s="10">
+      <c r="F19" s="10">
         <v>85</v>
       </c>
-      <c r="G18" s="10">
+      <c r="G19" s="10">
         <v>81</v>
       </c>
-      <c r="H18" s="10">
+      <c r="H19" s="10">
         <v>77</v>
       </c>
-      <c r="I18" s="10">
+      <c r="I19" s="10">
         <v>65</v>
       </c>
-      <c r="J18" s="10">
+      <c r="J19" s="10">
         <v>58</v>
       </c>
-      <c r="K18" s="10">
+      <c r="K19" s="10">
         <v>42</v>
       </c>
-      <c r="L18" s="10">
+      <c r="L19" s="10">
         <v>40</v>
       </c>
-      <c r="M18" s="10">
+      <c r="M19" s="10">
         <v>31</v>
       </c>
-      <c r="N18" s="10">
+      <c r="N19" s="10">
         <v>35</v>
       </c>
-    </row>
-    <row r="19" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B19" s="11" t="s">
+      <c r="P19" s="11" t="s">
+        <v>172</v>
+      </c>
+      <c r="Q19" s="10">
+        <v>0</v>
+      </c>
+      <c r="R19" s="10">
+        <v>72</v>
+      </c>
+      <c r="S19" s="10">
+        <v>78</v>
+      </c>
+      <c r="T19" s="10">
+        <v>70</v>
+      </c>
+      <c r="U19" s="10">
+        <v>85</v>
+      </c>
+      <c r="V19" s="10">
+        <v>80</v>
+      </c>
+      <c r="W19" s="10">
+        <v>55</v>
+      </c>
+      <c r="X19" s="10">
+        <v>40</v>
+      </c>
+      <c r="Y19" s="10">
+        <v>28</v>
+      </c>
+      <c r="Z19" s="10">
+        <v>52</v>
+      </c>
+      <c r="AA19" s="10">
+        <v>45</v>
+      </c>
+      <c r="AB19" s="10">
+        <v>50</v>
+      </c>
+      <c r="AD19" s="11" t="s">
+        <v>160</v>
+      </c>
+      <c r="AE19" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF19" s="10">
+        <v>92</v>
+      </c>
+      <c r="AG19" s="10">
+        <v>88</v>
+      </c>
+      <c r="AH19" s="10">
+        <v>95</v>
+      </c>
+      <c r="AI19" s="10">
+        <v>100</v>
+      </c>
+      <c r="AJ19" s="10">
+        <v>90</v>
+      </c>
+      <c r="AK19" s="10">
+        <v>72</v>
+      </c>
+      <c r="AL19" s="10">
+        <v>41</v>
+      </c>
+      <c r="AM19" s="10">
+        <v>33</v>
+      </c>
+      <c r="AN19" s="10">
+        <v>58</v>
+      </c>
+      <c r="AO19" s="10">
+        <v>54</v>
+      </c>
+      <c r="AP19" s="10">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="20" spans="2:42" x14ac:dyDescent="0.35">
+      <c r="B20" s="11" t="s">
         <v>161</v>
       </c>
-      <c r="C19" s="10">
+      <c r="C20" s="10">
         <v>96</v>
       </c>
-      <c r="D19" s="10">
+      <c r="D20" s="10">
         <v>0</v>
       </c>
-      <c r="E19" s="10">
+      <c r="E20" s="10">
         <v>89</v>
       </c>
-      <c r="F19" s="10">
+      <c r="F20" s="10">
         <v>83</v>
       </c>
-      <c r="G19" s="10">
+      <c r="G20" s="10">
         <v>78</v>
       </c>
-      <c r="H19" s="10">
+      <c r="H20" s="10">
         <v>75</v>
       </c>
-      <c r="I19" s="10">
+      <c r="I20" s="10">
         <v>60</v>
       </c>
-      <c r="J19" s="10">
+      <c r="J20" s="10">
         <v>63</v>
       </c>
-      <c r="K19" s="10">
+      <c r="K20" s="10">
         <v>38</v>
       </c>
-      <c r="L19" s="10">
+      <c r="L20" s="10">
         <v>51</v>
       </c>
-      <c r="M19" s="10">
+      <c r="M20" s="10">
         <v>33</v>
       </c>
-      <c r="N19" s="10">
+      <c r="N20" s="10">
         <v>29</v>
       </c>
-    </row>
-    <row r="20" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B20" s="11" t="s">
+      <c r="P20" s="11" t="s">
+        <v>161</v>
+      </c>
+      <c r="Q20" s="10">
+        <v>72</v>
+      </c>
+      <c r="R20" s="10">
+        <v>0</v>
+      </c>
+      <c r="S20" s="10">
+        <v>95</v>
+      </c>
+      <c r="T20" s="10">
+        <v>82</v>
+      </c>
+      <c r="U20" s="10">
+        <v>88</v>
+      </c>
+      <c r="V20" s="10">
+        <v>76</v>
+      </c>
+      <c r="W20" s="10">
+        <v>60</v>
+      </c>
+      <c r="X20" s="10">
+        <v>58</v>
+      </c>
+      <c r="Y20" s="10">
+        <v>42</v>
+      </c>
+      <c r="Z20" s="10">
+        <v>56</v>
+      </c>
+      <c r="AA20" s="10">
+        <v>54</v>
+      </c>
+      <c r="AB20" s="10">
+        <v>48</v>
+      </c>
+      <c r="AD20" s="11" t="s">
+        <v>161</v>
+      </c>
+      <c r="AE20" s="10">
+        <v>92</v>
+      </c>
+      <c r="AF20" s="10">
+        <v>0</v>
+      </c>
+      <c r="AG20" s="10">
+        <v>94</v>
+      </c>
+      <c r="AH20" s="10">
+        <v>89</v>
+      </c>
+      <c r="AI20" s="10">
+        <v>85</v>
+      </c>
+      <c r="AJ20" s="10">
+        <v>73</v>
+      </c>
+      <c r="AK20" s="10">
+        <v>57</v>
+      </c>
+      <c r="AL20" s="10">
+        <v>68</v>
+      </c>
+      <c r="AM20" s="10">
+        <v>49</v>
+      </c>
+      <c r="AN20" s="10">
+        <v>76</v>
+      </c>
+      <c r="AO20" s="10">
+        <v>46</v>
+      </c>
+      <c r="AP20" s="10">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="21" spans="2:42" x14ac:dyDescent="0.35">
+      <c r="B21" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="C20" s="10">
+      <c r="C21" s="10">
         <v>92</v>
       </c>
-      <c r="D20" s="10">
+      <c r="D21" s="10">
         <v>89</v>
       </c>
-      <c r="E20" s="10">
+      <c r="E21" s="10">
         <v>0</v>
       </c>
-      <c r="F20" s="10">
+      <c r="F21" s="10">
         <v>80</v>
       </c>
-      <c r="G20" s="10">
+      <c r="G21" s="10">
         <v>87</v>
       </c>
-      <c r="H20" s="10">
+      <c r="H21" s="10">
         <v>79</v>
       </c>
-      <c r="I20" s="10">
+      <c r="I21" s="10">
         <v>69</v>
       </c>
-      <c r="J20" s="10">
+      <c r="J21" s="10">
         <v>61</v>
       </c>
-      <c r="K20" s="10">
+      <c r="K21" s="10">
         <v>65</v>
       </c>
-      <c r="L20" s="10">
+      <c r="L21" s="10">
         <v>42</v>
       </c>
-      <c r="M20" s="10">
+      <c r="M21" s="10">
         <v>36</v>
       </c>
-      <c r="N20" s="10">
+      <c r="N21" s="10">
         <v>44</v>
       </c>
-    </row>
-    <row r="21" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B21" s="11" t="s">
+      <c r="P21" s="11" t="s">
+        <v>116</v>
+      </c>
+      <c r="Q21" s="10">
+        <v>78</v>
+      </c>
+      <c r="R21" s="10">
+        <v>95</v>
+      </c>
+      <c r="S21" s="10">
+        <v>0</v>
+      </c>
+      <c r="T21" s="10">
+        <v>84</v>
+      </c>
+      <c r="U21" s="10">
+        <v>90</v>
+      </c>
+      <c r="V21" s="10">
+        <v>82</v>
+      </c>
+      <c r="W21" s="10">
+        <v>65</v>
+      </c>
+      <c r="X21" s="10">
+        <v>62</v>
+      </c>
+      <c r="Y21" s="10">
+        <v>50</v>
+      </c>
+      <c r="Z21" s="10">
+        <v>48</v>
+      </c>
+      <c r="AA21" s="10">
+        <v>58</v>
+      </c>
+      <c r="AB21" s="10">
+        <v>57</v>
+      </c>
+      <c r="AD21" s="11" t="s">
+        <v>116</v>
+      </c>
+      <c r="AE21" s="10">
+        <v>88</v>
+      </c>
+      <c r="AF21" s="10">
+        <v>94</v>
+      </c>
+      <c r="AG21" s="10">
+        <v>0</v>
+      </c>
+      <c r="AH21" s="10">
+        <v>91</v>
+      </c>
+      <c r="AI21" s="10">
+        <v>87</v>
+      </c>
+      <c r="AJ21" s="10">
+        <v>79</v>
+      </c>
+      <c r="AK21" s="10">
+        <v>63</v>
+      </c>
+      <c r="AL21" s="10">
+        <v>52</v>
+      </c>
+      <c r="AM21" s="10">
+        <v>44</v>
+      </c>
+      <c r="AN21" s="10">
+        <v>71</v>
+      </c>
+      <c r="AO21" s="10">
+        <v>42</v>
+      </c>
+      <c r="AP21" s="10">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="22" spans="2:42" x14ac:dyDescent="0.35">
+      <c r="B22" s="11" t="s">
         <v>162</v>
       </c>
-      <c r="C21" s="10">
+      <c r="C22" s="10">
         <v>85</v>
       </c>
-      <c r="D21" s="10">
+      <c r="D22" s="10">
         <v>83</v>
       </c>
-      <c r="E21" s="10">
+      <c r="E22" s="10">
         <v>80</v>
       </c>
-      <c r="F21" s="10">
+      <c r="F22" s="10">
         <v>0</v>
       </c>
-      <c r="G21" s="10">
+      <c r="G22" s="10">
         <v>74</v>
       </c>
-      <c r="H21" s="10">
+      <c r="H22" s="10">
         <v>72</v>
       </c>
-      <c r="I21" s="10">
+      <c r="I22" s="10">
         <v>62</v>
       </c>
-      <c r="J21" s="10">
+      <c r="J22" s="10">
         <v>56</v>
       </c>
-      <c r="K21" s="10">
+      <c r="K22" s="10">
         <v>40</v>
       </c>
-      <c r="L21" s="10">
+      <c r="L22" s="10">
         <v>38</v>
       </c>
-      <c r="M21" s="10">
+      <c r="M22" s="10">
         <v>24</v>
       </c>
-      <c r="N21" s="10">
+      <c r="N22" s="10">
         <v>31</v>
       </c>
-    </row>
-    <row r="22" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B22" s="11" t="s">
+      <c r="P22" s="11" t="s">
+        <v>162</v>
+      </c>
+      <c r="Q22" s="10">
+        <v>70</v>
+      </c>
+      <c r="R22" s="10">
+        <v>82</v>
+      </c>
+      <c r="S22" s="10">
+        <v>84</v>
+      </c>
+      <c r="T22" s="10">
+        <v>0</v>
+      </c>
+      <c r="U22" s="10">
+        <v>86</v>
+      </c>
+      <c r="V22" s="10">
+        <v>74</v>
+      </c>
+      <c r="W22" s="10">
+        <v>53</v>
+      </c>
+      <c r="X22" s="10">
+        <v>64</v>
+      </c>
+      <c r="Y22" s="10">
+        <v>46</v>
+      </c>
+      <c r="Z22" s="10">
+        <v>44</v>
+      </c>
+      <c r="AA22" s="10">
+        <v>43</v>
+      </c>
+      <c r="AB22" s="10">
+        <v>41</v>
+      </c>
+      <c r="AD22" s="11" t="s">
+        <v>162</v>
+      </c>
+      <c r="AE22" s="10">
+        <v>95</v>
+      </c>
+      <c r="AF22" s="10">
+        <v>89</v>
+      </c>
+      <c r="AG22" s="10">
+        <v>91</v>
+      </c>
+      <c r="AH22" s="10">
+        <v>0</v>
+      </c>
+      <c r="AI22" s="10">
+        <v>96</v>
+      </c>
+      <c r="AJ22" s="10">
+        <v>84</v>
+      </c>
+      <c r="AK22" s="10">
+        <v>66</v>
+      </c>
+      <c r="AL22" s="10">
+        <v>61</v>
+      </c>
+      <c r="AM22" s="10">
+        <v>47</v>
+      </c>
+      <c r="AN22" s="10">
+        <v>74</v>
+      </c>
+      <c r="AO22" s="10">
+        <v>45</v>
+      </c>
+      <c r="AP22" s="10">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="23" spans="2:42" x14ac:dyDescent="0.35">
+      <c r="B23" s="11" t="s">
         <v>163</v>
       </c>
-      <c r="C22" s="10">
+      <c r="C23" s="10">
         <v>81</v>
       </c>
-      <c r="D22" s="10">
+      <c r="D23" s="10">
         <v>78</v>
       </c>
-      <c r="E22" s="10">
+      <c r="E23" s="10">
         <v>87</v>
       </c>
-      <c r="F22" s="10">
+      <c r="F23" s="10">
         <v>74</v>
       </c>
-      <c r="G22" s="10">
+      <c r="G23" s="10">
         <v>0</v>
       </c>
-      <c r="H22" s="10">
+      <c r="H23" s="10">
         <v>83</v>
       </c>
-      <c r="I22" s="10">
+      <c r="I23" s="10">
         <v>71</v>
       </c>
-      <c r="J22" s="10">
+      <c r="J23" s="10">
         <v>53</v>
       </c>
-      <c r="K22" s="10">
+      <c r="K23" s="10">
         <v>49</v>
       </c>
-      <c r="L22" s="10">
+      <c r="L23" s="10">
         <v>35</v>
       </c>
-      <c r="M22" s="10">
+      <c r="M23" s="10">
         <v>47</v>
       </c>
-      <c r="N22" s="10">
+      <c r="N23" s="10">
         <v>56</v>
       </c>
-    </row>
-    <row r="23" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B23" s="11" t="s">
+      <c r="P23" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="Q23" s="10">
+        <v>85</v>
+      </c>
+      <c r="R23" s="10">
+        <v>88</v>
+      </c>
+      <c r="S23" s="10">
+        <v>90</v>
+      </c>
+      <c r="T23" s="10">
+        <v>86</v>
+      </c>
+      <c r="U23" s="10">
+        <v>0</v>
+      </c>
+      <c r="V23" s="10">
+        <v>92</v>
+      </c>
+      <c r="W23" s="10">
+        <v>68</v>
+      </c>
+      <c r="X23" s="10">
+        <v>54</v>
+      </c>
+      <c r="Y23" s="10">
+        <v>38</v>
+      </c>
+      <c r="Z23" s="10">
+        <v>47</v>
+      </c>
+      <c r="AA23" s="10">
+        <v>75</v>
+      </c>
+      <c r="AB23" s="10">
+        <v>66</v>
+      </c>
+      <c r="AD23" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="AE23" s="10">
+        <v>100</v>
+      </c>
+      <c r="AF23" s="10">
+        <v>85</v>
+      </c>
+      <c r="AG23" s="10">
+        <v>87</v>
+      </c>
+      <c r="AH23" s="10">
+        <v>96</v>
+      </c>
+      <c r="AI23" s="10">
+        <v>0</v>
+      </c>
+      <c r="AJ23" s="10">
+        <v>93</v>
+      </c>
+      <c r="AK23" s="10">
+        <v>70</v>
+      </c>
+      <c r="AL23" s="10">
+        <v>43</v>
+      </c>
+      <c r="AM23" s="10">
+        <v>31</v>
+      </c>
+      <c r="AN23" s="10">
+        <v>56</v>
+      </c>
+      <c r="AO23" s="10">
+        <v>51</v>
+      </c>
+      <c r="AP23" s="10">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="24" spans="2:42" x14ac:dyDescent="0.35">
+      <c r="B24" s="11" t="s">
         <v>164</v>
       </c>
-      <c r="C23" s="10">
+      <c r="C24" s="10">
         <v>77</v>
       </c>
-      <c r="D23" s="10">
+      <c r="D24" s="10">
         <v>75</v>
       </c>
-      <c r="E23" s="10">
+      <c r="E24" s="10">
         <v>79</v>
       </c>
-      <c r="F23" s="10">
+      <c r="F24" s="10">
         <v>72</v>
       </c>
-      <c r="G23" s="10">
+      <c r="G24" s="10">
         <v>83</v>
       </c>
-      <c r="H23" s="10">
+      <c r="H24" s="10">
         <v>0</v>
       </c>
-      <c r="I23" s="10">
+      <c r="I24" s="10">
         <v>67</v>
       </c>
-      <c r="J23" s="10">
+      <c r="J24" s="10">
         <v>49</v>
       </c>
-      <c r="K23" s="10">
+      <c r="K24" s="10">
         <v>44</v>
       </c>
-      <c r="L23" s="10">
+      <c r="L24" s="10">
         <v>33</v>
       </c>
-      <c r="M23" s="10">
+      <c r="M24" s="10">
         <v>40</v>
       </c>
-      <c r="N23" s="10">
+      <c r="N24" s="10">
         <v>51</v>
       </c>
-    </row>
-    <row r="24" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B24" s="11" t="s">
+      <c r="P24" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="Q24" s="10">
+        <v>80</v>
+      </c>
+      <c r="R24" s="10">
+        <v>76</v>
+      </c>
+      <c r="S24" s="10">
+        <v>82</v>
+      </c>
+      <c r="T24" s="10">
+        <v>74</v>
+      </c>
+      <c r="U24" s="10">
+        <v>92</v>
+      </c>
+      <c r="V24" s="10">
+        <v>0</v>
+      </c>
+      <c r="W24" s="10">
+        <v>71</v>
+      </c>
+      <c r="X24" s="10">
+        <v>36</v>
+      </c>
+      <c r="Y24" s="10">
+        <v>34</v>
+      </c>
+      <c r="Z24" s="10">
+        <v>39</v>
+      </c>
+      <c r="AA24" s="10">
+        <v>67</v>
+      </c>
+      <c r="AB24" s="10">
+        <v>69</v>
+      </c>
+      <c r="AD24" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="AE24" s="10">
+        <v>90</v>
+      </c>
+      <c r="AF24" s="10">
+        <v>73</v>
+      </c>
+      <c r="AG24" s="10">
+        <v>79</v>
+      </c>
+      <c r="AH24" s="10">
+        <v>84</v>
+      </c>
+      <c r="AI24" s="10">
+        <v>93</v>
+      </c>
+      <c r="AJ24" s="10">
+        <v>0</v>
+      </c>
+      <c r="AK24" s="10">
+        <v>65</v>
+      </c>
+      <c r="AL24" s="10">
+        <v>36</v>
+      </c>
+      <c r="AM24" s="10">
+        <v>28</v>
+      </c>
+      <c r="AN24" s="10">
+        <v>48</v>
+      </c>
+      <c r="AO24" s="10">
+        <v>40</v>
+      </c>
+      <c r="AP24" s="10">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="25" spans="2:42" x14ac:dyDescent="0.35">
+      <c r="B25" s="11" t="s">
         <v>165</v>
       </c>
-      <c r="C24" s="10">
+      <c r="C25" s="10">
         <v>65</v>
       </c>
-      <c r="D24" s="10">
+      <c r="D25" s="10">
         <v>60</v>
       </c>
-      <c r="E24" s="10">
+      <c r="E25" s="10">
         <v>69</v>
       </c>
-      <c r="F24" s="10">
+      <c r="F25" s="10">
         <v>62</v>
       </c>
-      <c r="G24" s="10">
+      <c r="G25" s="10">
         <v>71</v>
       </c>
-      <c r="H24" s="10">
+      <c r="H25" s="10">
         <v>67</v>
       </c>
-      <c r="I24" s="10">
+      <c r="I25" s="10">
         <v>0</v>
       </c>
-      <c r="J24" s="10">
+      <c r="J25" s="10">
         <v>44</v>
       </c>
-      <c r="K24" s="10">
+      <c r="K25" s="10">
         <v>47</v>
       </c>
-      <c r="L24" s="10">
+      <c r="L25" s="10">
         <v>27</v>
       </c>
-      <c r="M24" s="10">
+      <c r="M25" s="10">
         <v>35</v>
       </c>
-      <c r="N24" s="10">
+      <c r="N25" s="10">
         <v>49</v>
       </c>
-    </row>
-    <row r="25" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B25" s="11" t="s">
+      <c r="P25" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="Q25" s="10">
+        <v>55</v>
+      </c>
+      <c r="R25" s="10">
+        <v>60</v>
+      </c>
+      <c r="S25" s="10">
+        <v>65</v>
+      </c>
+      <c r="T25" s="10">
+        <v>53</v>
+      </c>
+      <c r="U25" s="10">
+        <v>68</v>
+      </c>
+      <c r="V25" s="10">
+        <v>71</v>
+      </c>
+      <c r="W25" s="10">
+        <v>0</v>
+      </c>
+      <c r="X25" s="10">
+        <v>25</v>
+      </c>
+      <c r="Y25" s="10">
+        <v>30</v>
+      </c>
+      <c r="Z25" s="10">
+        <v>22</v>
+      </c>
+      <c r="AA25" s="10">
+        <v>49</v>
+      </c>
+      <c r="AB25" s="10">
+        <v>63</v>
+      </c>
+      <c r="AD25" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="AE25" s="10">
+        <v>72</v>
+      </c>
+      <c r="AF25" s="10">
+        <v>57</v>
+      </c>
+      <c r="AG25" s="10">
+        <v>63</v>
+      </c>
+      <c r="AH25" s="10">
+        <v>66</v>
+      </c>
+      <c r="AI25" s="10">
+        <v>70</v>
+      </c>
+      <c r="AJ25" s="10">
+        <v>65</v>
+      </c>
+      <c r="AK25" s="10">
+        <v>0</v>
+      </c>
+      <c r="AL25" s="10">
+        <v>22</v>
+      </c>
+      <c r="AM25" s="10">
+        <v>19</v>
+      </c>
+      <c r="AN25" s="10">
+        <v>34</v>
+      </c>
+      <c r="AO25" s="10">
+        <v>27</v>
+      </c>
+      <c r="AP25" s="10">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="26" spans="2:42" x14ac:dyDescent="0.35">
+      <c r="B26" s="11" t="s">
         <v>113</v>
       </c>
-      <c r="C25" s="10">
+      <c r="C26" s="10">
         <v>58</v>
       </c>
-      <c r="D25" s="10">
+      <c r="D26" s="10">
         <v>63</v>
       </c>
-      <c r="E25" s="10">
+      <c r="E26" s="10">
         <v>61</v>
       </c>
-      <c r="F25" s="10">
+      <c r="F26" s="10">
         <v>56</v>
       </c>
-      <c r="G25" s="10">
+      <c r="G26" s="10">
         <v>53</v>
       </c>
-      <c r="H25" s="10">
+      <c r="H26" s="10">
         <v>49</v>
       </c>
-      <c r="I25" s="10">
+      <c r="I26" s="10">
         <v>44</v>
       </c>
-      <c r="J25" s="10">
+      <c r="J26" s="10">
         <v>0</v>
       </c>
-      <c r="K25" s="10">
+      <c r="K26" s="10">
         <v>51</v>
       </c>
-      <c r="L25" s="10">
+      <c r="L26" s="10">
         <v>47</v>
       </c>
-      <c r="M25" s="10">
+      <c r="M26" s="10">
         <v>18</v>
       </c>
-      <c r="N25" s="10">
+      <c r="N26" s="10">
         <v>22</v>
       </c>
-    </row>
-    <row r="26" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B26" s="11" t="s">
+      <c r="P26" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="Q26" s="10">
+        <v>40</v>
+      </c>
+      <c r="R26" s="10">
+        <v>58</v>
+      </c>
+      <c r="S26" s="10">
+        <v>62</v>
+      </c>
+      <c r="T26" s="10">
+        <v>64</v>
+      </c>
+      <c r="U26" s="10">
+        <v>54</v>
+      </c>
+      <c r="V26" s="10">
+        <v>36</v>
+      </c>
+      <c r="W26" s="10">
+        <v>25</v>
+      </c>
+      <c r="X26" s="10">
+        <v>0</v>
+      </c>
+      <c r="Y26" s="10">
+        <v>26</v>
+      </c>
+      <c r="Z26" s="10">
+        <v>32</v>
+      </c>
+      <c r="AA26" s="10">
+        <v>18</v>
+      </c>
+      <c r="AB26" s="10">
+        <v>20</v>
+      </c>
+      <c r="AD26" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="AE26" s="10">
+        <v>41</v>
+      </c>
+      <c r="AF26" s="10">
+        <v>68</v>
+      </c>
+      <c r="AG26" s="10">
+        <v>52</v>
+      </c>
+      <c r="AH26" s="10">
+        <v>61</v>
+      </c>
+      <c r="AI26" s="10">
+        <v>43</v>
+      </c>
+      <c r="AJ26" s="10">
+        <v>36</v>
+      </c>
+      <c r="AK26" s="10">
+        <v>22</v>
+      </c>
+      <c r="AL26" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM26" s="10">
+        <v>17</v>
+      </c>
+      <c r="AN26" s="10">
+        <v>45</v>
+      </c>
+      <c r="AO26" s="10">
+        <v>12</v>
+      </c>
+      <c r="AP26" s="10">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="27" spans="2:42" x14ac:dyDescent="0.35">
+      <c r="B27" s="11" t="s">
         <v>120</v>
       </c>
-      <c r="C26" s="10">
+      <c r="C27" s="10">
         <v>42</v>
       </c>
-      <c r="D26" s="10">
+      <c r="D27" s="10">
         <v>38</v>
       </c>
-      <c r="E26" s="10">
+      <c r="E27" s="10">
         <v>65</v>
       </c>
-      <c r="F26" s="10">
+      <c r="F27" s="10">
         <v>40</v>
       </c>
-      <c r="G26" s="10">
+      <c r="G27" s="10">
         <v>49</v>
       </c>
-      <c r="H26" s="10">
+      <c r="H27" s="10">
         <v>44</v>
       </c>
-      <c r="I26" s="10">
+      <c r="I27" s="10">
         <v>47</v>
       </c>
-      <c r="J26" s="10">
+      <c r="J27" s="10">
         <v>51</v>
       </c>
-      <c r="K26" s="10">
+      <c r="K27" s="10">
         <v>0</v>
       </c>
-      <c r="L26" s="10">
+      <c r="L27" s="10">
         <v>31</v>
       </c>
-      <c r="M26" s="10">
+      <c r="M27" s="10">
         <v>15</v>
       </c>
-      <c r="N26" s="10">
+      <c r="N27" s="10">
         <v>27</v>
       </c>
-    </row>
-    <row r="27" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B27" s="11" t="s">
+      <c r="P27" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="Q27" s="10">
+        <v>28</v>
+      </c>
+      <c r="R27" s="10">
+        <v>42</v>
+      </c>
+      <c r="S27" s="10">
+        <v>50</v>
+      </c>
+      <c r="T27" s="10">
+        <v>46</v>
+      </c>
+      <c r="U27" s="10">
+        <v>38</v>
+      </c>
+      <c r="V27" s="10">
+        <v>34</v>
+      </c>
+      <c r="W27" s="10">
+        <v>30</v>
+      </c>
+      <c r="X27" s="10">
+        <v>26</v>
+      </c>
+      <c r="Y27" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z27" s="10">
+        <v>15</v>
+      </c>
+      <c r="AA27" s="10">
+        <v>12</v>
+      </c>
+      <c r="AB27" s="10">
+        <v>16</v>
+      </c>
+      <c r="AD27" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="AE27" s="10">
+        <v>33</v>
+      </c>
+      <c r="AF27" s="10">
+        <v>49</v>
+      </c>
+      <c r="AG27" s="10">
+        <v>44</v>
+      </c>
+      <c r="AH27" s="10">
+        <v>47</v>
+      </c>
+      <c r="AI27" s="10">
+        <v>31</v>
+      </c>
+      <c r="AJ27" s="10">
+        <v>28</v>
+      </c>
+      <c r="AK27" s="10">
+        <v>19</v>
+      </c>
+      <c r="AL27" s="10">
+        <v>17</v>
+      </c>
+      <c r="AM27" s="10">
+        <v>0</v>
+      </c>
+      <c r="AN27" s="10">
+        <v>29</v>
+      </c>
+      <c r="AO27" s="10">
+        <v>9</v>
+      </c>
+      <c r="AP27" s="10">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="28" spans="2:42" x14ac:dyDescent="0.35">
+      <c r="B28" s="11" t="s">
         <v>166</v>
       </c>
-      <c r="C27" s="10">
+      <c r="C28" s="10">
         <v>40</v>
       </c>
-      <c r="D27" s="10">
+      <c r="D28" s="10">
         <v>51</v>
       </c>
-      <c r="E27" s="10">
+      <c r="E28" s="10">
         <v>42</v>
       </c>
-      <c r="F27" s="10">
+      <c r="F28" s="10">
         <v>38</v>
       </c>
-      <c r="G27" s="10">
+      <c r="G28" s="10">
         <v>35</v>
       </c>
-      <c r="H27" s="10">
+      <c r="H28" s="10">
         <v>33</v>
       </c>
-      <c r="I27" s="10">
+      <c r="I28" s="10">
         <v>27</v>
       </c>
-      <c r="J27" s="10">
+      <c r="J28" s="10">
         <v>47</v>
       </c>
-      <c r="K27" s="10">
+      <c r="K28" s="10">
         <v>31</v>
       </c>
-      <c r="L27" s="10">
+      <c r="L28" s="10">
         <v>0</v>
       </c>
-      <c r="M27" s="10">
+      <c r="M28" s="10">
         <v>13</v>
       </c>
-      <c r="N27" s="10">
+      <c r="N28" s="10">
         <v>11</v>
       </c>
-    </row>
-    <row r="28" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B28" s="11" t="s">
+      <c r="P28" s="11" t="s">
+        <v>166</v>
+      </c>
+      <c r="Q28" s="10">
+        <v>52</v>
+      </c>
+      <c r="R28" s="10">
+        <v>56</v>
+      </c>
+      <c r="S28" s="10">
+        <v>48</v>
+      </c>
+      <c r="T28" s="10">
+        <v>44</v>
+      </c>
+      <c r="U28" s="10">
+        <v>47</v>
+      </c>
+      <c r="V28" s="10">
+        <v>39</v>
+      </c>
+      <c r="W28" s="10">
+        <v>22</v>
+      </c>
+      <c r="X28" s="10">
+        <v>32</v>
+      </c>
+      <c r="Y28" s="10">
+        <v>15</v>
+      </c>
+      <c r="Z28" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA28" s="10">
+        <v>14</v>
+      </c>
+      <c r="AB28" s="10">
+        <v>10</v>
+      </c>
+      <c r="AD28" s="11" t="s">
+        <v>174</v>
+      </c>
+      <c r="AE28" s="10">
+        <v>58</v>
+      </c>
+      <c r="AF28" s="10">
+        <v>76</v>
+      </c>
+      <c r="AG28" s="10">
+        <v>71</v>
+      </c>
+      <c r="AH28" s="10">
+        <v>74</v>
+      </c>
+      <c r="AI28" s="10">
+        <v>56</v>
+      </c>
+      <c r="AJ28" s="10">
+        <v>48</v>
+      </c>
+      <c r="AK28" s="10">
+        <v>34</v>
+      </c>
+      <c r="AL28" s="10">
+        <v>45</v>
+      </c>
+      <c r="AM28" s="10">
+        <v>29</v>
+      </c>
+      <c r="AN28" s="10">
+        <v>0</v>
+      </c>
+      <c r="AO28" s="10">
+        <v>26</v>
+      </c>
+      <c r="AP28" s="10">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="29" spans="2:42" x14ac:dyDescent="0.35">
+      <c r="B29" s="11" t="s">
         <v>167</v>
       </c>
-      <c r="C28" s="10">
+      <c r="C29" s="10">
         <v>31</v>
       </c>
-      <c r="D28" s="10">
+      <c r="D29" s="10">
         <v>33</v>
       </c>
-      <c r="E28" s="10">
+      <c r="E29" s="10">
         <v>36</v>
       </c>
-      <c r="F28" s="10">
+      <c r="F29" s="10">
         <v>24</v>
       </c>
-      <c r="G28" s="10">
+      <c r="G29" s="10">
         <v>47</v>
       </c>
-      <c r="H28" s="10">
+      <c r="H29" s="10">
         <v>40</v>
       </c>
-      <c r="I28" s="10">
+      <c r="I29" s="10">
         <v>35</v>
       </c>
-      <c r="J28" s="10">
+      <c r="J29" s="10">
         <v>18</v>
       </c>
-      <c r="K28" s="10">
+      <c r="K29" s="10">
         <v>15</v>
       </c>
-      <c r="L28" s="10">
+      <c r="L29" s="10">
         <v>13</v>
       </c>
-      <c r="M28" s="10">
+      <c r="M29" s="10">
         <v>0</v>
       </c>
-      <c r="N28" s="10">
+      <c r="N29" s="10">
         <v>42</v>
       </c>
-    </row>
-    <row r="29" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B29" s="11" t="s">
+      <c r="P29" s="11" t="s">
+        <v>167</v>
+      </c>
+      <c r="Q29" s="10">
+        <v>45</v>
+      </c>
+      <c r="R29" s="10">
+        <v>54</v>
+      </c>
+      <c r="S29" s="10">
+        <v>58</v>
+      </c>
+      <c r="T29" s="10">
+        <v>43</v>
+      </c>
+      <c r="U29" s="10">
+        <v>75</v>
+      </c>
+      <c r="V29" s="10">
+        <v>67</v>
+      </c>
+      <c r="W29" s="10">
+        <v>49</v>
+      </c>
+      <c r="X29" s="10">
+        <v>18</v>
+      </c>
+      <c r="Y29" s="10">
+        <v>12</v>
+      </c>
+      <c r="Z29" s="10">
+        <v>14</v>
+      </c>
+      <c r="AA29" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB29" s="10">
+        <v>24</v>
+      </c>
+      <c r="AD29" s="11" t="s">
+        <v>167</v>
+      </c>
+      <c r="AE29" s="10">
+        <v>54</v>
+      </c>
+      <c r="AF29" s="10">
+        <v>46</v>
+      </c>
+      <c r="AG29" s="10">
+        <v>42</v>
+      </c>
+      <c r="AH29" s="10">
+        <v>45</v>
+      </c>
+      <c r="AI29" s="10">
+        <v>51</v>
+      </c>
+      <c r="AJ29" s="10">
+        <v>40</v>
+      </c>
+      <c r="AK29" s="10">
+        <v>27</v>
+      </c>
+      <c r="AL29" s="10">
+        <v>12</v>
+      </c>
+      <c r="AM29" s="10">
+        <v>9</v>
+      </c>
+      <c r="AN29" s="10">
+        <v>26</v>
+      </c>
+      <c r="AO29" s="10">
+        <v>0</v>
+      </c>
+      <c r="AP29" s="10">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="30" spans="2:42" x14ac:dyDescent="0.35">
+      <c r="B30" s="11" t="s">
         <v>168</v>
       </c>
-      <c r="C29" s="10">
+      <c r="C30" s="10">
         <v>35</v>
       </c>
-      <c r="D29" s="10">
+      <c r="D30" s="10">
         <v>29</v>
       </c>
-      <c r="E29" s="10">
+      <c r="E30" s="10">
         <v>44</v>
       </c>
-      <c r="F29" s="10">
+      <c r="F30" s="10">
         <v>31</v>
       </c>
-      <c r="G29" s="10">
+      <c r="G30" s="10">
         <v>56</v>
       </c>
-      <c r="H29" s="10">
+      <c r="H30" s="10">
         <v>51</v>
       </c>
-      <c r="I29" s="10">
+      <c r="I30" s="10">
         <v>49</v>
       </c>
-      <c r="J29" s="10">
+      <c r="J30" s="10">
         <v>22</v>
       </c>
-      <c r="K29" s="10">
+      <c r="K30" s="10">
         <v>27</v>
       </c>
-      <c r="L29" s="10">
+      <c r="L30" s="10">
         <v>11</v>
       </c>
-      <c r="M29" s="10">
+      <c r="M30" s="10">
         <v>42</v>
       </c>
-      <c r="N29" s="10">
+      <c r="N30" s="10">
         <v>0</v>
       </c>
+      <c r="P30" s="11" t="s">
+        <v>168</v>
+      </c>
+      <c r="Q30" s="10">
+        <v>50</v>
+      </c>
+      <c r="R30" s="10">
+        <v>48</v>
+      </c>
+      <c r="S30" s="10">
+        <v>57</v>
+      </c>
+      <c r="T30" s="10">
+        <v>41</v>
+      </c>
+      <c r="U30" s="10">
+        <v>66</v>
+      </c>
+      <c r="V30" s="10">
+        <v>69</v>
+      </c>
+      <c r="W30" s="10">
+        <v>63</v>
+      </c>
+      <c r="X30" s="10">
+        <v>20</v>
+      </c>
+      <c r="Y30" s="10">
+        <v>16</v>
+      </c>
+      <c r="Z30" s="10">
+        <v>10</v>
+      </c>
+      <c r="AA30" s="10">
+        <v>24</v>
+      </c>
+      <c r="AB30" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD30" s="11" t="s">
+        <v>168</v>
+      </c>
+      <c r="AE30" s="10">
+        <v>61</v>
+      </c>
+      <c r="AF30" s="10">
+        <v>38</v>
+      </c>
+      <c r="AG30" s="10">
+        <v>35</v>
+      </c>
+      <c r="AH30" s="10">
+        <v>39</v>
+      </c>
+      <c r="AI30" s="10">
+        <v>59</v>
+      </c>
+      <c r="AJ30" s="10">
+        <v>67</v>
+      </c>
+      <c r="AK30" s="10">
+        <v>53</v>
+      </c>
+      <c r="AL30" s="10">
+        <v>24</v>
+      </c>
+      <c r="AM30" s="10">
+        <v>21</v>
+      </c>
+      <c r="AN30" s="10">
+        <v>32</v>
+      </c>
+      <c r="AO30" s="10">
+        <v>30</v>
+      </c>
+      <c r="AP30" s="10">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="C3:L12">
+  <conditionalFormatting sqref="C4:L13">
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C19:N30">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q4:Z13">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q19:AB30">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AE4:AN13">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -3995,7 +5801,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C18:N29">
+  <conditionalFormatting sqref="AE19:AP30">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>